<commit_message>
Refactor HMA solver: cleanup legacy benchmark files, translate comments to Vietnamese, add 30-run statistical comparison and update README documentation
</commit_message>
<xml_diff>
--- a/ketqua_hma.xlsx
+++ b/ketqua_hma.xlsx
@@ -6,14 +6,14 @@
     <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="LichTrinhHMA" r:id="rId5" sheetId="3"/>
-    <sheet name="HoiTu" r:id="rId6" sheetId="4"/>
+    <sheet name="LichTrinhHMA" r:id="rId4" sheetId="7"/>
+    <sheet name="HoiTu" r:id="rId5" sheetId="8"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="30">
   <si>
     <t>HMA TRANSPORTATION OPTIMIZATION PLAN</t>
   </si>
@@ -98,19 +98,37 @@
   <si>
     <t>Best Cost (TC)</t>
   </si>
+  <si>
+    <t>Total Cost (TC): 17.700.000 VND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - Operational Cost: 7.700.000 VND</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="9"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -161,7 +179,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
       <alignment horizontal="center"/>
@@ -172,13 +190,19 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
 </styleSheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="41.875" customWidth="true" bestFit="true"/>
@@ -197,7 +221,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3">
@@ -207,7 +231,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5">
@@ -216,25 +240,25 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="s" s="3">
+      <c r="A7" t="s" s="5">
         <v>5</v>
       </c>
-      <c r="B7" t="s" s="3">
+      <c r="B7" t="s" s="5">
         <v>6</v>
       </c>
-      <c r="C7" t="s" s="3">
+      <c r="C7" t="s" s="5">
         <v>7</v>
       </c>
-      <c r="D7" t="s" s="3">
+      <c r="D7" t="s" s="5">
         <v>8</v>
       </c>
-      <c r="E7" t="s" s="3">
+      <c r="E7" t="s" s="5">
         <v>9</v>
       </c>
-      <c r="F7" t="s" s="3">
+      <c r="F7" t="s" s="5">
         <v>10</v>
       </c>
-      <c r="G7" t="s" s="3">
+      <c r="G7" t="s" s="5">
         <v>11</v>
       </c>
     </row>
@@ -246,19 +270,19 @@
         <v>13</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D8" t="n" s="0">
-        <v>15.0</v>
+        <v>35.0</v>
       </c>
       <c r="E8" t="n" s="0">
-        <v>233.7821449197038</v>
+        <v>284.8162436403251</v>
       </c>
       <c r="F8" t="n" s="0">
-        <v>159.996875</v>
+        <v>133.75</v>
       </c>
       <c r="G8" t="n" s="0">
-        <v>450000.0</v>
+        <v>1400000.0</v>
       </c>
     </row>
     <row r="9">
@@ -269,50 +293,50 @@
         <v>15</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D9" t="n" s="0">
-        <v>25.0</v>
+        <v>15.0</v>
       </c>
       <c r="E9" t="n" s="0">
-        <v>308.7821449197038</v>
+        <v>209.81624364032513</v>
       </c>
       <c r="F9" t="n" s="0">
-        <v>159.99479166666666</v>
+        <v>148.75</v>
       </c>
       <c r="G9" t="n" s="0">
-        <v>900000.0</v>
+        <v>450000.0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D10" t="n" s="0">
-        <v>15.0</v>
+        <v>25.0</v>
       </c>
       <c r="E10" t="n" s="0">
-        <v>75.3637137846008</v>
+        <v>285.42297950765953</v>
       </c>
       <c r="F10" t="n" s="0">
-        <v>159.996875</v>
+        <v>141.25</v>
       </c>
       <c r="G10" t="n" s="0">
-        <v>450000.0</v>
+        <v>900000.0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="C11" t="s" s="0">
         <v>18</v>
@@ -321,10 +345,10 @@
         <v>15.0</v>
       </c>
       <c r="E11" t="n" s="0">
-        <v>158.7821449197038</v>
+        <v>0.0</v>
       </c>
       <c r="F11" t="n" s="0">
-        <v>159.996875</v>
+        <v>148.75</v>
       </c>
       <c r="G11" t="n" s="0">
         <v>450000.0</v>
@@ -335,68 +359,68 @@
         <v>19</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C12" t="s" s="0">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D12" t="n" s="0">
-        <v>35.0</v>
+        <v>15.0</v>
       </c>
       <c r="E12" t="n" s="0">
-        <v>238.50398295823</v>
+        <v>210.42297950765953</v>
       </c>
       <c r="F12" t="n" s="0">
-        <v>159.99270833333333</v>
+        <v>148.75</v>
       </c>
       <c r="G12" t="n" s="0">
-        <v>1400000.0</v>
+        <v>450000.0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D13" t="n" s="0">
-        <v>15.0</v>
+        <v>25.0</v>
       </c>
       <c r="E13" t="n" s="0">
-        <v>373.50398295823004</v>
+        <v>0.0</v>
       </c>
       <c r="F13" t="n" s="0">
-        <v>159.996875</v>
+        <v>141.25</v>
       </c>
       <c r="G13" t="n" s="0">
-        <v>450000.0</v>
+        <v>900000.0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C14" t="s" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D14" t="n" s="0">
-        <v>25.0</v>
+        <v>15.0</v>
       </c>
       <c r="E14" t="n" s="0">
-        <v>133.50398295823</v>
+        <v>283.8979374072738</v>
       </c>
       <c r="F14" t="n" s="0">
-        <v>159.99479166666666</v>
+        <v>148.75</v>
       </c>
       <c r="G14" t="n" s="0">
-        <v>900000.0</v>
+        <v>450000.0</v>
       </c>
     </row>
     <row r="15">
@@ -404,7 +428,7 @@
         <v>20</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C15" t="s" s="0">
         <v>16</v>
@@ -413,10 +437,10 @@
         <v>25.0</v>
       </c>
       <c r="E15" t="n" s="0">
-        <v>80.22613094691718</v>
+        <v>105.0</v>
       </c>
       <c r="F15" t="n" s="0">
-        <v>159.99479166666666</v>
+        <v>141.25</v>
       </c>
       <c r="G15" t="n" s="0">
         <v>900000.0</v>
@@ -424,162 +448,47 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C16" t="s" s="0">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D16" t="n" s="0">
-        <v>35.0</v>
+        <v>25.0</v>
       </c>
       <c r="E16" t="n" s="0">
-        <v>185.22613094691718</v>
+        <v>240.39254943241292</v>
       </c>
       <c r="F16" t="n" s="0">
-        <v>159.99270833333333</v>
+        <v>141.25</v>
       </c>
       <c r="G16" t="n" s="0">
-        <v>1400000.0</v>
+        <v>900000.0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C17" t="s" s="0">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D17" t="n" s="0">
-        <v>35.0</v>
+        <v>25.0</v>
       </c>
       <c r="E17" t="n" s="0">
-        <v>320.2261309469172</v>
+        <v>182.69699114683527</v>
       </c>
       <c r="F17" t="n" s="0">
-        <v>159.99270833333333</v>
+        <v>141.25</v>
       </c>
       <c r="G17" t="n" s="0">
-        <v>1400000.0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s" s="0">
-        <v>21</v>
-      </c>
-      <c r="B18" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="C18" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="D18" t="n" s="0">
-        <v>35.0</v>
-      </c>
-      <c r="E18" t="n" s="0">
-        <v>229.89956470357203</v>
-      </c>
-      <c r="F18" t="n" s="0">
-        <v>159.99270833333333</v>
-      </c>
-      <c r="G18" t="n" s="0">
-        <v>1400000.0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="s" s="0">
-        <v>21</v>
-      </c>
-      <c r="B19" t="s" s="0">
-        <v>15</v>
-      </c>
-      <c r="C19" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="D19" t="n" s="0">
-        <v>35.0</v>
-      </c>
-      <c r="E19" t="n" s="0">
-        <v>94.89956470357201</v>
-      </c>
-      <c r="F19" t="n" s="0">
-        <v>159.99270833333333</v>
-      </c>
-      <c r="G19" t="n" s="0">
-        <v>1400000.0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="B20" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="C20" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="D20" t="n" s="0">
-        <v>25.0</v>
-      </c>
-      <c r="E20" t="n" s="0">
-        <v>325.0904996617123</v>
-      </c>
-      <c r="F20" t="n" s="0">
-        <v>159.99479166666666</v>
-      </c>
-      <c r="G20" t="n" s="0">
-        <v>900000.0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="B21" t="s" s="0">
-        <v>15</v>
-      </c>
-      <c r="C21" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="D21" t="n" s="0">
-        <v>25.0</v>
-      </c>
-      <c r="E21" t="n" s="0">
-        <v>70.75430067673891</v>
-      </c>
-      <c r="F21" t="n" s="0">
-        <v>159.99479166666666</v>
-      </c>
-      <c r="G21" t="n" s="0">
-        <v>900000.0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="B22" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="C22" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="D22" t="n" s="0">
-        <v>25.0</v>
-      </c>
-      <c r="E22" t="n" s="0">
-        <v>220.09049966171227</v>
-      </c>
-      <c r="F22" t="n" s="0">
-        <v>159.99479166666666</v>
-      </c>
-      <c r="G22" t="n" s="0">
         <v>900000.0</v>
       </c>
     </row>
@@ -588,7 +497,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:B301"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
@@ -598,10 +507,10 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s" s="3">
+      <c r="A1" t="s" s="5">
         <v>26</v>
       </c>
-      <c r="B1" t="s" s="3">
+      <c r="B1" t="s" s="5">
         <v>27</v>
       </c>
     </row>
@@ -610,7 +519,7 @@
         <v>1.0</v>
       </c>
       <c r="B2" t="n" s="0">
-        <v>7.525E7</v>
+        <v>7.665E7</v>
       </c>
     </row>
     <row r="3">
@@ -618,7 +527,7 @@
         <v>2.0</v>
       </c>
       <c r="B3" t="n" s="0">
-        <v>7.47E7</v>
+        <v>9.34E7</v>
       </c>
     </row>
     <row r="4">
@@ -626,7 +535,7 @@
         <v>3.0</v>
       </c>
       <c r="B4" t="n" s="0">
-        <v>7.67E7</v>
+        <v>8.33E7</v>
       </c>
     </row>
     <row r="5">
@@ -634,7 +543,7 @@
         <v>4.0</v>
       </c>
       <c r="B5" t="n" s="0">
-        <v>8.285E7</v>
+        <v>8.43E7</v>
       </c>
     </row>
     <row r="6">
@@ -642,7 +551,7 @@
         <v>5.0</v>
       </c>
       <c r="B6" t="n" s="0">
-        <v>9.1E7</v>
+        <v>9.19E7</v>
       </c>
     </row>
     <row r="7">
@@ -650,7 +559,7 @@
         <v>6.0</v>
       </c>
       <c r="B7" t="n" s="0">
-        <v>8.33E7</v>
+        <v>8.675E7</v>
       </c>
     </row>
     <row r="8">
@@ -658,7 +567,7 @@
         <v>7.0</v>
       </c>
       <c r="B8" t="n" s="0">
-        <v>7.62E7</v>
+        <v>8.24E7</v>
       </c>
     </row>
     <row r="9">
@@ -666,7 +575,7 @@
         <v>8.0</v>
       </c>
       <c r="B9" t="n" s="0">
-        <v>8.63E7</v>
+        <v>1.0765E8</v>
       </c>
     </row>
     <row r="10">
@@ -674,7 +583,7 @@
         <v>9.0</v>
       </c>
       <c r="B10" t="n" s="0">
-        <v>7.06E7</v>
+        <v>8.19E7</v>
       </c>
     </row>
     <row r="11">
@@ -682,7 +591,7 @@
         <v>10.0</v>
       </c>
       <c r="B11" t="n" s="0">
-        <v>8.285E7</v>
+        <v>8.335E7</v>
       </c>
     </row>
     <row r="12">
@@ -690,7 +599,7 @@
         <v>11.0</v>
       </c>
       <c r="B12" t="n" s="0">
-        <v>7.67E7</v>
+        <v>8.425E7</v>
       </c>
     </row>
     <row r="13">
@@ -706,7 +615,7 @@
         <v>13.0</v>
       </c>
       <c r="B14" t="n" s="0">
-        <v>8.335E7</v>
+        <v>9.145E7</v>
       </c>
     </row>
     <row r="15">
@@ -714,7 +623,7 @@
         <v>14.0</v>
       </c>
       <c r="B15" t="n" s="0">
-        <v>7.475E7</v>
+        <v>7.42E7</v>
       </c>
     </row>
     <row r="16">
@@ -722,7 +631,7 @@
         <v>15.0</v>
       </c>
       <c r="B16" t="n" s="0">
-        <v>7.375E7</v>
+        <v>9.145E7</v>
       </c>
     </row>
     <row r="17">
@@ -730,7 +639,7 @@
         <v>16.0</v>
       </c>
       <c r="B17" t="n" s="0">
-        <v>7.625E7</v>
+        <v>8.19E7</v>
       </c>
     </row>
     <row r="18">
@@ -738,7 +647,7 @@
         <v>17.0</v>
       </c>
       <c r="B18" t="n" s="0">
-        <v>6.67E7</v>
+        <v>8.33E7</v>
       </c>
     </row>
     <row r="19">
@@ -746,7 +655,7 @@
         <v>18.0</v>
       </c>
       <c r="B19" t="n" s="0">
-        <v>7.475E7</v>
+        <v>9.195E7</v>
       </c>
     </row>
     <row r="20">
@@ -754,7 +663,7 @@
         <v>19.0</v>
       </c>
       <c r="B20" t="n" s="0">
-        <v>8.43E7</v>
+        <v>9.24E7</v>
       </c>
     </row>
     <row r="21">
@@ -762,7 +671,7 @@
         <v>20.0</v>
       </c>
       <c r="B21" t="n" s="0">
-        <v>8.725E7</v>
+        <v>9.095E7</v>
       </c>
     </row>
     <row r="22">
@@ -770,7 +679,7 @@
         <v>21.0</v>
       </c>
       <c r="B22" t="n" s="0">
-        <v>8.38E7</v>
+        <v>8.28E7</v>
       </c>
     </row>
     <row r="23">
@@ -778,7 +687,7 @@
         <v>22.0</v>
       </c>
       <c r="B23" t="n" s="0">
-        <v>7.725E7</v>
+        <v>8.285E7</v>
       </c>
     </row>
     <row r="24">
@@ -786,7 +695,7 @@
         <v>23.0</v>
       </c>
       <c r="B24" t="n" s="0">
-        <v>7.72E7</v>
+        <v>1.0195E8</v>
       </c>
     </row>
     <row r="25">
@@ -794,7 +703,7 @@
         <v>24.0</v>
       </c>
       <c r="B25" t="n" s="0">
-        <v>8.235E7</v>
+        <v>1.0195E8</v>
       </c>
     </row>
     <row r="26">
@@ -802,7 +711,7 @@
         <v>25.0</v>
       </c>
       <c r="B26" t="n" s="0">
-        <v>7.47E7</v>
+        <v>6.905E7</v>
       </c>
     </row>
     <row r="27">
@@ -810,7 +719,7 @@
         <v>26.0</v>
       </c>
       <c r="B27" t="n" s="0">
-        <v>8.285E7</v>
+        <v>7.575E7</v>
       </c>
     </row>
     <row r="28">
@@ -818,7 +727,7 @@
         <v>27.0</v>
       </c>
       <c r="B28" t="n" s="0">
-        <v>8.38E7</v>
+        <v>8.335E7</v>
       </c>
     </row>
     <row r="29">
@@ -826,7 +735,7 @@
         <v>28.0</v>
       </c>
       <c r="B29" t="n" s="0">
-        <v>8.535E7</v>
+        <v>7.72E7</v>
       </c>
     </row>
     <row r="30">
@@ -834,7 +743,7 @@
         <v>29.0</v>
       </c>
       <c r="B30" t="n" s="0">
-        <v>9.85E7</v>
+        <v>9.195E7</v>
       </c>
     </row>
     <row r="31">
@@ -842,7 +751,7 @@
         <v>30.0</v>
       </c>
       <c r="B31" t="n" s="0">
-        <v>5.855E7</v>
+        <v>8.485E7</v>
       </c>
     </row>
     <row r="32">
@@ -850,7 +759,7 @@
         <v>31.0</v>
       </c>
       <c r="B32" t="n" s="0">
-        <v>7.33E7</v>
+        <v>8.63E7</v>
       </c>
     </row>
     <row r="33">
@@ -858,7 +767,7 @@
         <v>32.0</v>
       </c>
       <c r="B33" t="n" s="0">
-        <v>6.005E7</v>
+        <v>9.145E7</v>
       </c>
     </row>
     <row r="34">
@@ -866,7 +775,7 @@
         <v>33.0</v>
       </c>
       <c r="B34" t="n" s="0">
-        <v>7.575E7</v>
+        <v>8.58E7</v>
       </c>
     </row>
     <row r="35">
@@ -874,7 +783,7 @@
         <v>34.0</v>
       </c>
       <c r="B35" t="n" s="0">
-        <v>8.28E7</v>
+        <v>8.33E7</v>
       </c>
     </row>
     <row r="36">
@@ -882,7 +791,7 @@
         <v>35.0</v>
       </c>
       <c r="B36" t="n" s="0">
-        <v>5.805E7</v>
+        <v>6.57E7</v>
       </c>
     </row>
     <row r="37">
@@ -890,7 +799,7 @@
         <v>36.0</v>
       </c>
       <c r="B37" t="n" s="0">
-        <v>7.575E7</v>
+        <v>7.62E7</v>
       </c>
     </row>
     <row r="38">
@@ -898,7 +807,7 @@
         <v>37.0</v>
       </c>
       <c r="B38" t="n" s="0">
-        <v>7.325E7</v>
+        <v>7.675E7</v>
       </c>
     </row>
     <row r="39">
@@ -906,7 +815,7 @@
         <v>38.0</v>
       </c>
       <c r="B39" t="n" s="0">
-        <v>7.625E7</v>
+        <v>7.675E7</v>
       </c>
     </row>
     <row r="40">
@@ -914,7 +823,7 @@
         <v>39.0</v>
       </c>
       <c r="B40" t="n" s="0">
-        <v>8.425E7</v>
+        <v>8.33E7</v>
       </c>
     </row>
     <row r="41">
@@ -922,7 +831,7 @@
         <v>40.0</v>
       </c>
       <c r="B41" t="n" s="0">
-        <v>8.38E7</v>
+        <v>9.39E7</v>
       </c>
     </row>
     <row r="42">
@@ -930,7 +839,7 @@
         <v>41.0</v>
       </c>
       <c r="B42" t="n" s="0">
-        <v>7.67E7</v>
+        <v>7.325E7</v>
       </c>
     </row>
     <row r="43">
@@ -938,7 +847,7 @@
         <v>42.0</v>
       </c>
       <c r="B43" t="n" s="0">
-        <v>6.67E7</v>
+        <v>8.38E7</v>
       </c>
     </row>
     <row r="44">
@@ -946,7 +855,7 @@
         <v>43.0</v>
       </c>
       <c r="B44" t="n" s="0">
-        <v>8.53E7</v>
+        <v>8.28E7</v>
       </c>
     </row>
     <row r="45">
@@ -954,7 +863,7 @@
         <v>44.0</v>
       </c>
       <c r="B45" t="n" s="0">
-        <v>8.38E7</v>
+        <v>8.28E7</v>
       </c>
     </row>
     <row r="46">
@@ -962,7 +871,7 @@
         <v>45.0</v>
       </c>
       <c r="B46" t="n" s="0">
-        <v>8.285E7</v>
+        <v>6.76E7</v>
       </c>
     </row>
     <row r="47">
@@ -970,7 +879,7 @@
         <v>46.0</v>
       </c>
       <c r="B47" t="n" s="0">
-        <v>8.675E7</v>
+        <v>7.375E7</v>
       </c>
     </row>
     <row r="48">
@@ -978,7 +887,7 @@
         <v>47.0</v>
       </c>
       <c r="B48" t="n" s="0">
-        <v>5.9E7</v>
+        <v>7.375E7</v>
       </c>
     </row>
     <row r="49">
@@ -986,7 +895,7 @@
         <v>48.0</v>
       </c>
       <c r="B49" t="n" s="0">
-        <v>7.67E7</v>
+        <v>6.57E7</v>
       </c>
     </row>
     <row r="50">
@@ -994,7 +903,7 @@
         <v>49.0</v>
       </c>
       <c r="B50" t="n" s="0">
-        <v>8.335E7</v>
+        <v>6.865E7</v>
       </c>
     </row>
     <row r="51">
@@ -1002,7 +911,7 @@
         <v>50.0</v>
       </c>
       <c r="B51" t="n" s="0">
-        <v>8.33E7</v>
+        <v>7.43E7</v>
       </c>
     </row>
     <row r="52">
@@ -1010,7 +919,7 @@
         <v>51.0</v>
       </c>
       <c r="B52" t="n" s="0">
-        <v>7.42E7</v>
+        <v>6.77E7</v>
       </c>
     </row>
     <row r="53">
@@ -1018,7 +927,7 @@
         <v>52.0</v>
       </c>
       <c r="B53" t="n" s="0">
-        <v>8.0E7</v>
+        <v>6.57E7</v>
       </c>
     </row>
     <row r="54">
@@ -1026,7 +935,7 @@
         <v>53.0</v>
       </c>
       <c r="B54" t="n" s="0">
-        <v>7.77E7</v>
+        <v>6.61E7</v>
       </c>
     </row>
     <row r="55">
@@ -1034,7 +943,7 @@
         <v>54.0</v>
       </c>
       <c r="B55" t="n" s="0">
-        <v>6.81E7</v>
+        <v>6.57E7</v>
       </c>
     </row>
     <row r="56">
@@ -1042,7 +951,7 @@
         <v>55.0</v>
       </c>
       <c r="B56" t="n" s="0">
-        <v>7.525E7</v>
+        <v>6.37E7</v>
       </c>
     </row>
     <row r="57">
@@ -1050,7 +959,7 @@
         <v>56.0</v>
       </c>
       <c r="B57" t="n" s="0">
-        <v>8.235E7</v>
+        <v>6.62E7</v>
       </c>
     </row>
     <row r="58">
@@ -1058,7 +967,7 @@
         <v>57.0</v>
       </c>
       <c r="B58" t="n" s="0">
-        <v>6.86E7</v>
+        <v>7.575E7</v>
       </c>
     </row>
     <row r="59">
@@ -1066,7 +975,7 @@
         <v>58.0</v>
       </c>
       <c r="B59" t="n" s="0">
-        <v>7.33E7</v>
+        <v>6.715E7</v>
       </c>
     </row>
     <row r="60">
@@ -1074,7 +983,7 @@
         <v>59.0</v>
       </c>
       <c r="B60" t="n" s="0">
-        <v>7.62E7</v>
+        <v>9.24E7</v>
       </c>
     </row>
     <row r="61">
@@ -1082,7 +991,7 @@
         <v>60.0</v>
       </c>
       <c r="B61" t="n" s="0">
-        <v>5.855E7</v>
+        <v>9.145E7</v>
       </c>
     </row>
     <row r="62">
@@ -1090,7 +999,7 @@
         <v>61.0</v>
       </c>
       <c r="B62" t="n" s="0">
-        <v>7.28E7</v>
+        <v>6.71E7</v>
       </c>
     </row>
     <row r="63">
@@ -1098,7 +1007,7 @@
         <v>62.0</v>
       </c>
       <c r="B63" t="n" s="0">
-        <v>6.62E7</v>
+        <v>9.1E7</v>
       </c>
     </row>
     <row r="64">
@@ -1106,7 +1015,7 @@
         <v>63.0</v>
       </c>
       <c r="B64" t="n" s="0">
-        <v>6.81E7</v>
+        <v>8.235E7</v>
       </c>
     </row>
     <row r="65">
@@ -1114,7 +1023,7 @@
         <v>64.0</v>
       </c>
       <c r="B65" t="n" s="0">
-        <v>7.375E7</v>
+        <v>6.415E7</v>
       </c>
     </row>
     <row r="66">
@@ -1122,7 +1031,7 @@
         <v>65.0</v>
       </c>
       <c r="B66" t="n" s="0">
-        <v>6.62E7</v>
+        <v>6.67E7</v>
       </c>
     </row>
     <row r="67">
@@ -1130,7 +1039,7 @@
         <v>66.0</v>
       </c>
       <c r="B67" t="n" s="0">
-        <v>7.575E7</v>
+        <v>7.375E7</v>
       </c>
     </row>
     <row r="68">
@@ -1138,7 +1047,7 @@
         <v>67.0</v>
       </c>
       <c r="B68" t="n" s="0">
-        <v>6.665E7</v>
+        <v>4.945E7</v>
       </c>
     </row>
     <row r="69">
@@ -1146,7 +1055,7 @@
         <v>68.0</v>
       </c>
       <c r="B69" t="n" s="0">
-        <v>5.755E7</v>
+        <v>7.375E7</v>
       </c>
     </row>
     <row r="70">
@@ -1154,7 +1063,7 @@
         <v>69.0</v>
       </c>
       <c r="B70" t="n" s="0">
-        <v>5.71E7</v>
+        <v>7.625E7</v>
       </c>
     </row>
     <row r="71">
@@ -1162,7 +1071,7 @@
         <v>70.0</v>
       </c>
       <c r="B71" t="n" s="0">
-        <v>6.865E7</v>
+        <v>7.375E7</v>
       </c>
     </row>
     <row r="72">
@@ -1170,7 +1079,7 @@
         <v>71.0</v>
       </c>
       <c r="B72" t="n" s="0">
-        <v>5.1E7</v>
+        <v>7.67E7</v>
       </c>
     </row>
     <row r="73">
@@ -1178,7 +1087,7 @@
         <v>72.0</v>
       </c>
       <c r="B73" t="n" s="0">
-        <v>6.515E7</v>
+        <v>6.865E7</v>
       </c>
     </row>
     <row r="74">
@@ -1186,7 +1095,7 @@
         <v>73.0</v>
       </c>
       <c r="B74" t="n" s="0">
-        <v>5.905E7</v>
+        <v>7.33E7</v>
       </c>
     </row>
     <row r="75">
@@ -1194,7 +1103,7 @@
         <v>74.0</v>
       </c>
       <c r="B75" t="n" s="0">
-        <v>7.67E7</v>
+        <v>6.665E7</v>
       </c>
     </row>
     <row r="76">
@@ -1202,7 +1111,7 @@
         <v>75.0</v>
       </c>
       <c r="B76" t="n" s="0">
-        <v>7.245E7</v>
+        <v>6.42E7</v>
       </c>
     </row>
     <row r="77">
@@ -1210,7 +1119,7 @@
         <v>76.0</v>
       </c>
       <c r="B77" t="n" s="0">
-        <v>7.015E7</v>
+        <v>6.715E7</v>
       </c>
     </row>
     <row r="78">
@@ -1218,7 +1127,7 @@
         <v>77.0</v>
       </c>
       <c r="B78" t="n" s="0">
-        <v>6.055E7</v>
+        <v>6.05E7</v>
       </c>
     </row>
     <row r="79">
@@ -1226,7 +1135,7 @@
         <v>78.0</v>
       </c>
       <c r="B79" t="n" s="0">
-        <v>7.575E7</v>
+        <v>5.71E7</v>
       </c>
     </row>
     <row r="80">
@@ -1234,7 +1143,7 @@
         <v>79.0</v>
       </c>
       <c r="B80" t="n" s="0">
-        <v>6.62E7</v>
+        <v>6.42E7</v>
       </c>
     </row>
     <row r="81">
@@ -1242,7 +1151,7 @@
         <v>80.0</v>
       </c>
       <c r="B81" t="n" s="0">
-        <v>6.86E7</v>
+        <v>7.325E7</v>
       </c>
     </row>
     <row r="82">
@@ -1258,7 +1167,7 @@
         <v>82.0</v>
       </c>
       <c r="B83" t="n" s="0">
-        <v>6.005E7</v>
+        <v>5.855E7</v>
       </c>
     </row>
     <row r="84">
@@ -1266,7 +1175,7 @@
         <v>83.0</v>
       </c>
       <c r="B84" t="n" s="0">
-        <v>5.95E7</v>
+        <v>6.42E7</v>
       </c>
     </row>
     <row r="85">
@@ -1274,7 +1183,7 @@
         <v>84.0</v>
       </c>
       <c r="B85" t="n" s="0">
-        <v>5.755E7</v>
+        <v>7.525E7</v>
       </c>
     </row>
     <row r="86">
@@ -1282,7 +1191,7 @@
         <v>85.0</v>
       </c>
       <c r="B86" t="n" s="0">
-        <v>6.81E7</v>
+        <v>7.42E7</v>
       </c>
     </row>
     <row r="87">
@@ -1298,7 +1207,7 @@
         <v>87.0</v>
       </c>
       <c r="B88" t="n" s="0">
-        <v>6.105E7</v>
+        <v>6.665E7</v>
       </c>
     </row>
     <row r="89">
@@ -1306,7 +1215,7 @@
         <v>88.0</v>
       </c>
       <c r="B89" t="n" s="0">
-        <v>5.76E7</v>
+        <v>5.855E7</v>
       </c>
     </row>
     <row r="90">
@@ -1314,7 +1223,7 @@
         <v>89.0</v>
       </c>
       <c r="B90" t="n" s="0">
-        <v>6.715E7</v>
+        <v>6.615E7</v>
       </c>
     </row>
     <row r="91">
@@ -1322,7 +1231,7 @@
         <v>90.0</v>
       </c>
       <c r="B91" t="n" s="0">
-        <v>6.715E7</v>
+        <v>6.15E7</v>
       </c>
     </row>
     <row r="92">
@@ -1330,7 +1239,7 @@
         <v>91.0</v>
       </c>
       <c r="B92" t="n" s="0">
-        <v>6.105E7</v>
+        <v>8.335E7</v>
       </c>
     </row>
     <row r="93">
@@ -1338,7 +1247,7 @@
         <v>92.0</v>
       </c>
       <c r="B93" t="n" s="0">
-        <v>5.855E7</v>
+        <v>8.29E7</v>
       </c>
     </row>
     <row r="94">
@@ -1346,7 +1255,7 @@
         <v>93.0</v>
       </c>
       <c r="B94" t="n" s="0">
-        <v>4.995E7</v>
+        <v>7.62E7</v>
       </c>
     </row>
     <row r="95">
@@ -1354,7 +1263,7 @@
         <v>94.0</v>
       </c>
       <c r="B95" t="n" s="0">
-        <v>6.615E7</v>
+        <v>5.71E7</v>
       </c>
     </row>
     <row r="96">
@@ -1362,7 +1271,7 @@
         <v>95.0</v>
       </c>
       <c r="B96" t="n" s="0">
-        <v>6.715E7</v>
+        <v>6.42E7</v>
       </c>
     </row>
     <row r="97">
@@ -1370,7 +1279,7 @@
         <v>96.0</v>
       </c>
       <c r="B97" t="n" s="0">
-        <v>8.335E7</v>
+        <v>5.81E7</v>
       </c>
     </row>
     <row r="98">
@@ -1378,7 +1287,7 @@
         <v>97.0</v>
       </c>
       <c r="B98" t="n" s="0">
-        <v>4.895E7</v>
+        <v>5.85E7</v>
       </c>
     </row>
     <row r="99">
@@ -1386,7 +1295,7 @@
         <v>98.0</v>
       </c>
       <c r="B99" t="n" s="0">
-        <v>7.38E7</v>
+        <v>5.9E7</v>
       </c>
     </row>
     <row r="100">
@@ -1394,7 +1303,7 @@
         <v>99.0</v>
       </c>
       <c r="B100" t="n" s="0">
-        <v>6.76E7</v>
+        <v>5.855E7</v>
       </c>
     </row>
     <row r="101">
@@ -1402,7 +1311,7 @@
         <v>100.0</v>
       </c>
       <c r="B101" t="n" s="0">
-        <v>5.805E7</v>
+        <v>6.57E7</v>
       </c>
     </row>
     <row r="102">
@@ -1410,7 +1319,7 @@
         <v>101.0</v>
       </c>
       <c r="B102" t="n" s="0">
-        <v>6.86E7</v>
+        <v>6.62E7</v>
       </c>
     </row>
     <row r="103">
@@ -1418,7 +1327,7 @@
         <v>102.0</v>
       </c>
       <c r="B103" t="n" s="0">
-        <v>6.615E7</v>
+        <v>6.62E7</v>
       </c>
     </row>
     <row r="104">
@@ -1426,7 +1335,7 @@
         <v>103.0</v>
       </c>
       <c r="B104" t="n" s="0">
-        <v>7.62E7</v>
+        <v>4.24E7</v>
       </c>
     </row>
     <row r="105">
@@ -1434,7 +1343,7 @@
         <v>104.0</v>
       </c>
       <c r="B105" t="n" s="0">
-        <v>8.33E7</v>
+        <v>6.515E7</v>
       </c>
     </row>
     <row r="106">
@@ -1442,7 +1351,7 @@
         <v>105.0</v>
       </c>
       <c r="B106" t="n" s="0">
-        <v>7.475E7</v>
+        <v>5.76E7</v>
       </c>
     </row>
     <row r="107">
@@ -1450,7 +1359,7 @@
         <v>106.0</v>
       </c>
       <c r="B107" t="n" s="0">
-        <v>7.525E7</v>
+        <v>6.715E7</v>
       </c>
     </row>
     <row r="108">
@@ -1458,7 +1367,7 @@
         <v>107.0</v>
       </c>
       <c r="B108" t="n" s="0">
-        <v>8.0E7</v>
+        <v>6.76E7</v>
       </c>
     </row>
     <row r="109">
@@ -1466,7 +1375,7 @@
         <v>108.0</v>
       </c>
       <c r="B109" t="n" s="0">
-        <v>6.765E7</v>
+        <v>5.76E7</v>
       </c>
     </row>
     <row r="110">
@@ -1474,7 +1383,7 @@
         <v>109.0</v>
       </c>
       <c r="B110" t="n" s="0">
-        <v>6.71E7</v>
+        <v>6.62E7</v>
       </c>
     </row>
     <row r="111">
@@ -1490,7 +1399,7 @@
         <v>111.0</v>
       </c>
       <c r="B112" t="n" s="0">
-        <v>6.715E7</v>
+        <v>7.425E7</v>
       </c>
     </row>
     <row r="113">
@@ -1498,7 +1407,7 @@
         <v>112.0</v>
       </c>
       <c r="B113" t="n" s="0">
-        <v>5.855E7</v>
+        <v>5.95E7</v>
       </c>
     </row>
     <row r="114">
@@ -1506,7 +1415,7 @@
         <v>113.0</v>
       </c>
       <c r="B114" t="n" s="0">
-        <v>6.81E7</v>
+        <v>6.57E7</v>
       </c>
     </row>
     <row r="115">
@@ -1514,7 +1423,7 @@
         <v>114.0</v>
       </c>
       <c r="B115" t="n" s="0">
-        <v>5.805E7</v>
+        <v>6.76E7</v>
       </c>
     </row>
     <row r="116">
@@ -1522,7 +1431,7 @@
         <v>115.0</v>
       </c>
       <c r="B116" t="n" s="0">
-        <v>5.755E7</v>
+        <v>6.1E7</v>
       </c>
     </row>
     <row r="117">
@@ -1530,7 +1439,7 @@
         <v>116.0</v>
       </c>
       <c r="B117" t="n" s="0">
-        <v>6.615E7</v>
+        <v>5.71E7</v>
       </c>
     </row>
     <row r="118">
@@ -1538,7 +1447,7 @@
         <v>117.0</v>
       </c>
       <c r="B118" t="n" s="0">
-        <v>6.81E7</v>
+        <v>4.19E7</v>
       </c>
     </row>
     <row r="119">
@@ -1546,7 +1455,7 @@
         <v>118.0</v>
       </c>
       <c r="B119" t="n" s="0">
-        <v>7.52E7</v>
+        <v>5.91E7</v>
       </c>
     </row>
     <row r="120">
@@ -1554,7 +1463,7 @@
         <v>119.0</v>
       </c>
       <c r="B120" t="n" s="0">
-        <v>6.71E7</v>
+        <v>5.24E7</v>
       </c>
     </row>
     <row r="121">
@@ -1562,7 +1471,7 @@
         <v>120.0</v>
       </c>
       <c r="B121" t="n" s="0">
-        <v>5.66E7</v>
+        <v>5.1E7</v>
       </c>
     </row>
     <row r="122">
@@ -1570,7 +1479,7 @@
         <v>121.0</v>
       </c>
       <c r="B122" t="n" s="0">
-        <v>5.905E7</v>
+        <v>6.77E7</v>
       </c>
     </row>
     <row r="123">
@@ -1578,7 +1487,7 @@
         <v>122.0</v>
       </c>
       <c r="B123" t="n" s="0">
-        <v>5.805E7</v>
+        <v>5.86E7</v>
       </c>
     </row>
     <row r="124">
@@ -1586,7 +1495,7 @@
         <v>123.0</v>
       </c>
       <c r="B124" t="n" s="0">
-        <v>6.71E7</v>
+        <v>7.375E7</v>
       </c>
     </row>
     <row r="125">
@@ -1594,7 +1503,7 @@
         <v>124.0</v>
       </c>
       <c r="B125" t="n" s="0">
-        <v>4.085E7</v>
+        <v>7.375E7</v>
       </c>
     </row>
     <row r="126">
@@ -1602,7 +1511,7 @@
         <v>125.0</v>
       </c>
       <c r="B126" t="n" s="0">
-        <v>5.81E7</v>
+        <v>7.575E7</v>
       </c>
     </row>
     <row r="127">
@@ -1610,7 +1519,7 @@
         <v>126.0</v>
       </c>
       <c r="B127" t="n" s="0">
-        <v>4.945E7</v>
+        <v>5.15E7</v>
       </c>
     </row>
     <row r="128">
@@ -1618,7 +1527,7 @@
         <v>127.0</v>
       </c>
       <c r="B128" t="n" s="0">
-        <v>7.525E7</v>
+        <v>5.91E7</v>
       </c>
     </row>
     <row r="129">
@@ -1626,7 +1535,7 @@
         <v>128.0</v>
       </c>
       <c r="B129" t="n" s="0">
-        <v>4.945E7</v>
+        <v>6.815E7</v>
       </c>
     </row>
     <row r="130">
@@ -1634,7 +1543,7 @@
         <v>129.0</v>
       </c>
       <c r="B130" t="n" s="0">
-        <v>6.665E7</v>
+        <v>7.525E7</v>
       </c>
     </row>
     <row r="131">
@@ -1642,7 +1551,7 @@
         <v>130.0</v>
       </c>
       <c r="B131" t="n" s="0">
-        <v>6.42E7</v>
+        <v>5.195E7</v>
       </c>
     </row>
     <row r="132">
@@ -1650,7 +1559,7 @@
         <v>131.0</v>
       </c>
       <c r="B132" t="n" s="0">
-        <v>5.755E7</v>
+        <v>4.24E7</v>
       </c>
     </row>
     <row r="133">
@@ -1658,7 +1567,7 @@
         <v>132.0</v>
       </c>
       <c r="B133" t="n" s="0">
-        <v>5.855E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="134">
@@ -1666,7 +1575,7 @@
         <v>133.0</v>
       </c>
       <c r="B134" t="n" s="0">
-        <v>5.755E7</v>
+        <v>5.145E7</v>
       </c>
     </row>
     <row r="135">
@@ -1674,7 +1583,7 @@
         <v>134.0</v>
       </c>
       <c r="B135" t="n" s="0">
-        <v>4.895E7</v>
+        <v>5.145E7</v>
       </c>
     </row>
     <row r="136">
@@ -1682,7 +1591,7 @@
         <v>135.0</v>
       </c>
       <c r="B136" t="n" s="0">
-        <v>5.04E7</v>
+        <v>5.91E7</v>
       </c>
     </row>
     <row r="137">
@@ -1690,7 +1599,7 @@
         <v>136.0</v>
       </c>
       <c r="B137" t="n" s="0">
-        <v>4.945E7</v>
+        <v>6.86E7</v>
       </c>
     </row>
     <row r="138">
@@ -1698,7 +1607,7 @@
         <v>137.0</v>
       </c>
       <c r="B138" t="n" s="0">
-        <v>5.855E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="139">
@@ -1706,7 +1615,7 @@
         <v>138.0</v>
       </c>
       <c r="B139" t="n" s="0">
-        <v>5.855E7</v>
+        <v>5.19E7</v>
       </c>
     </row>
     <row r="140">
@@ -1714,7 +1623,7 @@
         <v>139.0</v>
       </c>
       <c r="B140" t="n" s="0">
-        <v>5.805E7</v>
+        <v>6.665E7</v>
       </c>
     </row>
     <row r="141">
@@ -1722,7 +1631,7 @@
         <v>140.0</v>
       </c>
       <c r="B141" t="n" s="0">
-        <v>4.995E7</v>
+        <v>7.29E7</v>
       </c>
     </row>
     <row r="142">
@@ -1730,7 +1639,7 @@
         <v>141.0</v>
       </c>
       <c r="B142" t="n" s="0">
-        <v>4.995E7</v>
+        <v>6.77E7</v>
       </c>
     </row>
     <row r="143">
@@ -1738,7 +1647,7 @@
         <v>142.0</v>
       </c>
       <c r="B143" t="n" s="0">
-        <v>4.085E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="144">
@@ -1746,7 +1655,7 @@
         <v>143.0</v>
       </c>
       <c r="B144" t="n" s="0">
-        <v>4.85E7</v>
+        <v>5.195E7</v>
       </c>
     </row>
     <row r="145">
@@ -1754,7 +1663,7 @@
         <v>144.0</v>
       </c>
       <c r="B145" t="n" s="0">
-        <v>4.04E7</v>
+        <v>5.05E7</v>
       </c>
     </row>
     <row r="146">
@@ -1762,7 +1671,7 @@
         <v>145.0</v>
       </c>
       <c r="B146" t="n" s="0">
-        <v>4.515E7</v>
+        <v>5.195E7</v>
       </c>
     </row>
     <row r="147">
@@ -1770,7 +1679,7 @@
         <v>146.0</v>
       </c>
       <c r="B147" t="n" s="0">
-        <v>6.855E7</v>
+        <v>5.1E7</v>
       </c>
     </row>
     <row r="148">
@@ -1778,7 +1687,7 @@
         <v>147.0</v>
       </c>
       <c r="B148" t="n" s="0">
-        <v>6.905E7</v>
+        <v>5.71E7</v>
       </c>
     </row>
     <row r="149">
@@ -1786,7 +1695,7 @@
         <v>148.0</v>
       </c>
       <c r="B149" t="n" s="0">
-        <v>5.755E7</v>
+        <v>5.1E7</v>
       </c>
     </row>
     <row r="150">
@@ -1794,7 +1703,7 @@
         <v>149.0</v>
       </c>
       <c r="B150" t="n" s="0">
-        <v>3.94E7</v>
+        <v>6.715E7</v>
       </c>
     </row>
     <row r="151">
@@ -1802,7 +1711,7 @@
         <v>150.0</v>
       </c>
       <c r="B151" t="n" s="0">
-        <v>3.94E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="152">
@@ -1810,7 +1719,7 @@
         <v>151.0</v>
       </c>
       <c r="B152" t="n" s="0">
-        <v>4.895E7</v>
+        <v>4.285E7</v>
       </c>
     </row>
     <row r="153">
@@ -1818,7 +1727,7 @@
         <v>152.0</v>
       </c>
       <c r="B153" t="n" s="0">
-        <v>3.99E7</v>
+        <v>5.85E7</v>
       </c>
     </row>
     <row r="154">
@@ -1826,7 +1735,7 @@
         <v>153.0</v>
       </c>
       <c r="B154" t="n" s="0">
-        <v>4.85E7</v>
+        <v>6.57E7</v>
       </c>
     </row>
     <row r="155">
@@ -1834,7 +1743,7 @@
         <v>154.0</v>
       </c>
       <c r="B155" t="n" s="0">
-        <v>4.895E7</v>
+        <v>5.095E7</v>
       </c>
     </row>
     <row r="156">
@@ -1842,7 +1751,7 @@
         <v>155.0</v>
       </c>
       <c r="B156" t="n" s="0">
-        <v>4.085E7</v>
+        <v>5.86E7</v>
       </c>
     </row>
     <row r="157">
@@ -1850,7 +1759,7 @@
         <v>156.0</v>
       </c>
       <c r="B157" t="n" s="0">
-        <v>3.99E7</v>
+        <v>5.145E7</v>
       </c>
     </row>
     <row r="158">
@@ -1858,7 +1767,7 @@
         <v>157.0</v>
       </c>
       <c r="B158" t="n" s="0">
-        <v>4.85E7</v>
+        <v>5.095E7</v>
       </c>
     </row>
     <row r="159">
@@ -1866,7 +1775,7 @@
         <v>158.0</v>
       </c>
       <c r="B159" t="n" s="0">
-        <v>3.94E7</v>
+        <v>5.1E7</v>
       </c>
     </row>
     <row r="160">
@@ -1874,7 +1783,7 @@
         <v>159.0</v>
       </c>
       <c r="B160" t="n" s="0">
-        <v>4.035E7</v>
+        <v>4.285E7</v>
       </c>
     </row>
     <row r="161">
@@ -1882,7 +1791,7 @@
         <v>160.0</v>
       </c>
       <c r="B161" t="n" s="0">
-        <v>3.99E7</v>
+        <v>4.285E7</v>
       </c>
     </row>
     <row r="162">
@@ -1890,7 +1799,7 @@
         <v>161.0</v>
       </c>
       <c r="B162" t="n" s="0">
-        <v>4.995E7</v>
+        <v>6.15E7</v>
       </c>
     </row>
     <row r="163">
@@ -1898,7 +1807,7 @@
         <v>162.0</v>
       </c>
       <c r="B163" t="n" s="0">
-        <v>4.04E7</v>
+        <v>4.285E7</v>
       </c>
     </row>
     <row r="164">
@@ -1906,7 +1815,7 @@
         <v>163.0</v>
       </c>
       <c r="B164" t="n" s="0">
-        <v>4.04E7</v>
+        <v>4.285E7</v>
       </c>
     </row>
     <row r="165">
@@ -1914,7 +1823,7 @@
         <v>164.0</v>
       </c>
       <c r="B165" t="n" s="0">
-        <v>3.99E7</v>
+        <v>5.145E7</v>
       </c>
     </row>
     <row r="166">
@@ -1922,7 +1831,7 @@
         <v>165.0</v>
       </c>
       <c r="B166" t="n" s="0">
-        <v>3.94E7</v>
+        <v>6.665E7</v>
       </c>
     </row>
     <row r="167">
@@ -1930,7 +1839,7 @@
         <v>166.0</v>
       </c>
       <c r="B167" t="n" s="0">
-        <v>4.85E7</v>
+        <v>5.145E7</v>
       </c>
     </row>
     <row r="168">
@@ -1938,7 +1847,7 @@
         <v>167.0</v>
       </c>
       <c r="B168" t="n" s="0">
-        <v>3.94E7</v>
+        <v>5.195E7</v>
       </c>
     </row>
     <row r="169">
@@ -1946,7 +1855,7 @@
         <v>168.0</v>
       </c>
       <c r="B169" t="n" s="0">
-        <v>4.04E7</v>
+        <v>4.19E7</v>
       </c>
     </row>
     <row r="170">
@@ -1954,7 +1863,7 @@
         <v>169.0</v>
       </c>
       <c r="B170" t="n" s="0">
-        <v>4.85E7</v>
+        <v>5.195E7</v>
       </c>
     </row>
     <row r="171">
@@ -1962,7 +1871,7 @@
         <v>170.0</v>
       </c>
       <c r="B171" t="n" s="0">
-        <v>4.04E7</v>
+        <v>5.19E7</v>
       </c>
     </row>
     <row r="172">
@@ -1970,7 +1879,7 @@
         <v>171.0</v>
       </c>
       <c r="B172" t="n" s="0">
-        <v>4.04E7</v>
+        <v>5.1E7</v>
       </c>
     </row>
     <row r="173">
@@ -1978,7 +1887,7 @@
         <v>172.0</v>
       </c>
       <c r="B173" t="n" s="0">
-        <v>3.94E7</v>
+        <v>5.05E7</v>
       </c>
     </row>
     <row r="174">
@@ -1986,7 +1895,7 @@
         <v>173.0</v>
       </c>
       <c r="B174" t="n" s="0">
-        <v>3.94E7</v>
+        <v>4.19E7</v>
       </c>
     </row>
     <row r="175">
@@ -1994,7 +1903,7 @@
         <v>174.0</v>
       </c>
       <c r="B175" t="n" s="0">
-        <v>4.9E7</v>
+        <v>6.665E7</v>
       </c>
     </row>
     <row r="176">
@@ -2002,7 +1911,7 @@
         <v>175.0</v>
       </c>
       <c r="B176" t="n" s="0">
-        <v>3.94E7</v>
+        <v>5.1E7</v>
       </c>
     </row>
     <row r="177">
@@ -2010,7 +1919,7 @@
         <v>176.0</v>
       </c>
       <c r="B177" t="n" s="0">
-        <v>3.94E7</v>
+        <v>4.285E7</v>
       </c>
     </row>
     <row r="178">
@@ -2018,7 +1927,7 @@
         <v>177.0</v>
       </c>
       <c r="B178" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.285E7</v>
       </c>
     </row>
     <row r="179">
@@ -2026,7 +1935,7 @@
         <v>178.0</v>
       </c>
       <c r="B179" t="n" s="0">
-        <v>3.94E7</v>
+        <v>4.19E7</v>
       </c>
     </row>
     <row r="180">
@@ -2034,7 +1943,7 @@
         <v>179.0</v>
       </c>
       <c r="B180" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.19E7</v>
       </c>
     </row>
     <row r="181">
@@ -2042,7 +1951,7 @@
         <v>180.0</v>
       </c>
       <c r="B181" t="n" s="0">
-        <v>3.56E7</v>
+        <v>5.145E7</v>
       </c>
     </row>
     <row r="182">
@@ -2050,7 +1959,7 @@
         <v>181.0</v>
       </c>
       <c r="B182" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.235E7</v>
       </c>
     </row>
     <row r="183">
@@ -2058,7 +1967,7 @@
         <v>182.0</v>
       </c>
       <c r="B183" t="n" s="0">
-        <v>3.375E7</v>
+        <v>5.095E7</v>
       </c>
     </row>
     <row r="184">
@@ -2066,7 +1975,7 @@
         <v>183.0</v>
       </c>
       <c r="B184" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.19E7</v>
       </c>
     </row>
     <row r="185">
@@ -2074,7 +1983,7 @@
         <v>184.0</v>
       </c>
       <c r="B185" t="n" s="0">
-        <v>3.56E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="186">
@@ -2082,7 +1991,7 @@
         <v>185.0</v>
       </c>
       <c r="B186" t="n" s="0">
-        <v>3.375E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="187">
@@ -2090,7 +1999,7 @@
         <v>186.0</v>
       </c>
       <c r="B187" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.195E7</v>
       </c>
     </row>
     <row r="188">
@@ -2098,7 +2007,7 @@
         <v>187.0</v>
       </c>
       <c r="B188" t="n" s="0">
-        <v>4.035E7</v>
+        <v>5.145E7</v>
       </c>
     </row>
     <row r="189">
@@ -2106,7 +2015,7 @@
         <v>188.0</v>
       </c>
       <c r="B189" t="n" s="0">
-        <v>3.33E7</v>
+        <v>4.235E7</v>
       </c>
     </row>
     <row r="190">
@@ -2114,7 +2023,7 @@
         <v>189.0</v>
       </c>
       <c r="B190" t="n" s="0">
-        <v>3.33E7</v>
+        <v>5.1E7</v>
       </c>
     </row>
     <row r="191">
@@ -2122,7 +2031,7 @@
         <v>190.0</v>
       </c>
       <c r="B191" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="192">
@@ -2130,7 +2039,7 @@
         <v>191.0</v>
       </c>
       <c r="B192" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.235E7</v>
       </c>
     </row>
     <row r="193">
@@ -2138,7 +2047,7 @@
         <v>192.0</v>
       </c>
       <c r="B193" t="n" s="0">
-        <v>4.085E7</v>
+        <v>5.195E7</v>
       </c>
     </row>
     <row r="194">
@@ -2146,7 +2055,7 @@
         <v>193.0</v>
       </c>
       <c r="B194" t="n" s="0">
-        <v>3.375E7</v>
+        <v>6.815E7</v>
       </c>
     </row>
     <row r="195">
@@ -2154,7 +2063,7 @@
         <v>194.0</v>
       </c>
       <c r="B195" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.285E7</v>
       </c>
     </row>
     <row r="196">
@@ -2162,7 +2071,7 @@
         <v>195.0</v>
       </c>
       <c r="B196" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.24E7</v>
       </c>
     </row>
     <row r="197">
@@ -2170,7 +2079,7 @@
         <v>196.0</v>
       </c>
       <c r="B197" t="n" s="0">
-        <v>3.375E7</v>
+        <v>6.15E7</v>
       </c>
     </row>
     <row r="198">
@@ -2178,7 +2087,7 @@
         <v>197.0</v>
       </c>
       <c r="B198" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.05E7</v>
       </c>
     </row>
     <row r="199">
@@ -2186,7 +2095,7 @@
         <v>198.0</v>
       </c>
       <c r="B199" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.145E7</v>
       </c>
     </row>
     <row r="200">
@@ -2194,7 +2103,7 @@
         <v>199.0</v>
       </c>
       <c r="B200" t="n" s="0">
-        <v>3.375E7</v>
+        <v>4.235E7</v>
       </c>
     </row>
     <row r="201">
@@ -2202,7 +2111,7 @@
         <v>200.0</v>
       </c>
       <c r="B201" t="n" s="0">
-        <v>3.375E7</v>
+        <v>5.05E7</v>
       </c>
     </row>
     <row r="202">
@@ -2210,7 +2119,7 @@
         <v>201.0</v>
       </c>
       <c r="B202" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="203">
@@ -2218,7 +2127,7 @@
         <v>202.0</v>
       </c>
       <c r="B203" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.145E7</v>
       </c>
     </row>
     <row r="204">
@@ -2226,7 +2135,7 @@
         <v>203.0</v>
       </c>
       <c r="B204" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="205">
@@ -2234,7 +2143,7 @@
         <v>204.0</v>
       </c>
       <c r="B205" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.05E7</v>
       </c>
     </row>
     <row r="206">
@@ -2242,7 +2151,7 @@
         <v>205.0</v>
       </c>
       <c r="B206" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.285E7</v>
       </c>
     </row>
     <row r="207">
@@ -2250,7 +2159,7 @@
         <v>206.0</v>
       </c>
       <c r="B207" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.145E7</v>
       </c>
     </row>
     <row r="208">
@@ -2258,7 +2167,7 @@
         <v>207.0</v>
       </c>
       <c r="B208" t="n" s="0">
-        <v>3.33E7</v>
+        <v>4.24E7</v>
       </c>
     </row>
     <row r="209">
@@ -2266,7 +2175,7 @@
         <v>208.0</v>
       </c>
       <c r="B209" t="n" s="0">
-        <v>3.56E7</v>
+        <v>4.285E7</v>
       </c>
     </row>
     <row r="210">
@@ -2274,7 +2183,7 @@
         <v>209.0</v>
       </c>
       <c r="B210" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.19E7</v>
       </c>
     </row>
     <row r="211">
@@ -2282,7 +2191,7 @@
         <v>210.0</v>
       </c>
       <c r="B211" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.24E7</v>
       </c>
     </row>
     <row r="212">
@@ -2290,7 +2199,7 @@
         <v>211.0</v>
       </c>
       <c r="B212" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="213">
@@ -2298,7 +2207,7 @@
         <v>212.0</v>
       </c>
       <c r="B213" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.19E7</v>
       </c>
     </row>
     <row r="214">
@@ -2306,7 +2215,7 @@
         <v>213.0</v>
       </c>
       <c r="B214" t="n" s="0">
-        <v>3.33E7</v>
+        <v>4.19E7</v>
       </c>
     </row>
     <row r="215">
@@ -2314,7 +2223,7 @@
         <v>214.0</v>
       </c>
       <c r="B215" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.24E7</v>
       </c>
     </row>
     <row r="216">
@@ -2322,7 +2231,7 @@
         <v>215.0</v>
       </c>
       <c r="B216" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="217">
@@ -2330,7 +2239,7 @@
         <v>216.0</v>
       </c>
       <c r="B217" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.05E7</v>
       </c>
     </row>
     <row r="218">
@@ -2338,7 +2247,7 @@
         <v>217.0</v>
       </c>
       <c r="B218" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.1E7</v>
       </c>
     </row>
     <row r="219">
@@ -2346,7 +2255,7 @@
         <v>218.0</v>
       </c>
       <c r="B219" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.235E7</v>
       </c>
     </row>
     <row r="220">
@@ -2354,7 +2263,7 @@
         <v>219.0</v>
       </c>
       <c r="B220" t="n" s="0">
-        <v>3.94E7</v>
+        <v>4.19E7</v>
       </c>
     </row>
     <row r="221">
@@ -2362,7 +2271,7 @@
         <v>220.0</v>
       </c>
       <c r="B221" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.05E7</v>
       </c>
     </row>
     <row r="222">
@@ -2370,7 +2279,7 @@
         <v>221.0</v>
       </c>
       <c r="B222" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.19E7</v>
       </c>
     </row>
     <row r="223">
@@ -2378,7 +2287,7 @@
         <v>222.0</v>
       </c>
       <c r="B223" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.19E7</v>
       </c>
     </row>
     <row r="224">
@@ -2386,7 +2295,7 @@
         <v>223.0</v>
       </c>
       <c r="B224" t="n" s="0">
-        <v>3.33E7</v>
+        <v>5.05E7</v>
       </c>
     </row>
     <row r="225">
@@ -2394,7 +2303,7 @@
         <v>224.0</v>
       </c>
       <c r="B225" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.33E7</v>
       </c>
     </row>
     <row r="226">
@@ -2402,7 +2311,7 @@
         <v>225.0</v>
       </c>
       <c r="B226" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="227">
@@ -2410,7 +2319,7 @@
         <v>226.0</v>
       </c>
       <c r="B227" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.05E7</v>
       </c>
     </row>
     <row r="228">
@@ -2418,7 +2327,7 @@
         <v>227.0</v>
       </c>
       <c r="B228" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="229">
@@ -2426,7 +2335,7 @@
         <v>228.0</v>
       </c>
       <c r="B229" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.19E7</v>
       </c>
     </row>
     <row r="230">
@@ -2434,7 +2343,7 @@
         <v>229.0</v>
       </c>
       <c r="B230" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="231">
@@ -2442,7 +2351,7 @@
         <v>230.0</v>
       </c>
       <c r="B231" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.145E7</v>
       </c>
     </row>
     <row r="232">
@@ -2450,7 +2359,7 @@
         <v>231.0</v>
       </c>
       <c r="B232" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.05E7</v>
       </c>
     </row>
     <row r="233">
@@ -2458,7 +2367,7 @@
         <v>232.0</v>
       </c>
       <c r="B233" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="234">
@@ -2466,7 +2375,7 @@
         <v>233.0</v>
       </c>
       <c r="B234" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="235">
@@ -2474,7 +2383,7 @@
         <v>234.0</v>
       </c>
       <c r="B235" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="236">
@@ -2482,7 +2391,7 @@
         <v>235.0</v>
       </c>
       <c r="B236" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.195E7</v>
       </c>
     </row>
     <row r="237">
@@ -2490,7 +2399,7 @@
         <v>236.0</v>
       </c>
       <c r="B237" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.285E7</v>
       </c>
     </row>
     <row r="238">
@@ -2498,7 +2407,7 @@
         <v>237.0</v>
       </c>
       <c r="B238" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="239">
@@ -2506,7 +2415,7 @@
         <v>238.0</v>
       </c>
       <c r="B239" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.05E7</v>
       </c>
     </row>
     <row r="240">
@@ -2514,7 +2423,7 @@
         <v>239.0</v>
       </c>
       <c r="B240" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="241">
@@ -2522,7 +2431,7 @@
         <v>240.0</v>
       </c>
       <c r="B241" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.285E7</v>
       </c>
     </row>
     <row r="242">
@@ -2530,7 +2439,7 @@
         <v>241.0</v>
       </c>
       <c r="B242" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.235E7</v>
       </c>
     </row>
     <row r="243">
@@ -2538,7 +2447,7 @@
         <v>242.0</v>
       </c>
       <c r="B243" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.19E7</v>
       </c>
     </row>
     <row r="244">
@@ -2546,7 +2455,7 @@
         <v>243.0</v>
       </c>
       <c r="B244" t="n" s="0">
-        <v>3.08E7</v>
+        <v>4.19E7</v>
       </c>
     </row>
     <row r="245">
@@ -2554,7 +2463,7 @@
         <v>244.0</v>
       </c>
       <c r="B245" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.19E7</v>
       </c>
     </row>
     <row r="246">
@@ -2562,7 +2471,7 @@
         <v>245.0</v>
       </c>
       <c r="B246" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="247">
@@ -2570,7 +2479,7 @@
         <v>246.0</v>
       </c>
       <c r="B247" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.05E7</v>
       </c>
     </row>
     <row r="248">
@@ -2578,7 +2487,7 @@
         <v>247.0</v>
       </c>
       <c r="B248" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.1E7</v>
       </c>
     </row>
     <row r="249">
@@ -2586,7 +2495,7 @@
         <v>248.0</v>
       </c>
       <c r="B249" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.285E7</v>
       </c>
     </row>
     <row r="250">
@@ -2594,7 +2503,7 @@
         <v>249.0</v>
       </c>
       <c r="B250" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.19E7</v>
       </c>
     </row>
     <row r="251">
@@ -2602,7 +2511,7 @@
         <v>250.0</v>
       </c>
       <c r="B251" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="252">
@@ -2610,7 +2519,7 @@
         <v>251.0</v>
       </c>
       <c r="B252" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="253">
@@ -2618,7 +2527,7 @@
         <v>252.0</v>
       </c>
       <c r="B253" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="254">
@@ -2626,7 +2535,7 @@
         <v>253.0</v>
       </c>
       <c r="B254" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.145E7</v>
       </c>
     </row>
     <row r="255">
@@ -2634,7 +2543,7 @@
         <v>254.0</v>
       </c>
       <c r="B255" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="256">
@@ -2642,7 +2551,7 @@
         <v>255.0</v>
       </c>
       <c r="B256" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="257">
@@ -2650,7 +2559,7 @@
         <v>256.0</v>
       </c>
       <c r="B257" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.28E7</v>
       </c>
     </row>
     <row r="258">
@@ -2658,7 +2567,7 @@
         <v>257.0</v>
       </c>
       <c r="B258" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.47E7</v>
       </c>
     </row>
     <row r="259">
@@ -2666,7 +2575,7 @@
         <v>258.0</v>
       </c>
       <c r="B259" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.76E7</v>
       </c>
     </row>
     <row r="260">
@@ -2674,7 +2583,7 @@
         <v>259.0</v>
       </c>
       <c r="B260" t="n" s="0">
-        <v>2.42E7</v>
+        <v>6.62E7</v>
       </c>
     </row>
     <row r="261">
@@ -2682,7 +2591,7 @@
         <v>260.0</v>
       </c>
       <c r="B261" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.19E7</v>
       </c>
     </row>
     <row r="262">
@@ -2690,7 +2599,7 @@
         <v>261.0</v>
       </c>
       <c r="B262" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.235E7</v>
       </c>
     </row>
     <row r="263">
@@ -2698,7 +2607,7 @@
         <v>262.0</v>
       </c>
       <c r="B263" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.285E7</v>
       </c>
     </row>
     <row r="264">
@@ -2706,7 +2615,7 @@
         <v>263.0</v>
       </c>
       <c r="B264" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.285E7</v>
       </c>
     </row>
     <row r="265">
@@ -2714,7 +2623,7 @@
         <v>264.0</v>
       </c>
       <c r="B265" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.285E7</v>
       </c>
     </row>
     <row r="266">
@@ -2722,7 +2631,7 @@
         <v>265.0</v>
       </c>
       <c r="B266" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.19E7</v>
       </c>
     </row>
     <row r="267">
@@ -2730,7 +2639,7 @@
         <v>266.0</v>
       </c>
       <c r="B267" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.05E7</v>
       </c>
     </row>
     <row r="268">
@@ -2738,7 +2647,7 @@
         <v>267.0</v>
       </c>
       <c r="B268" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.28E7</v>
       </c>
     </row>
     <row r="269">
@@ -2746,7 +2655,7 @@
         <v>268.0</v>
       </c>
       <c r="B269" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.375E7</v>
       </c>
     </row>
     <row r="270">
@@ -2754,7 +2663,7 @@
         <v>269.0</v>
       </c>
       <c r="B270" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.28E7</v>
       </c>
     </row>
     <row r="271">
@@ -2762,7 +2671,7 @@
         <v>270.0</v>
       </c>
       <c r="B271" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.375E7</v>
       </c>
     </row>
     <row r="272">
@@ -2770,7 +2679,7 @@
         <v>271.0</v>
       </c>
       <c r="B272" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.375E7</v>
       </c>
     </row>
     <row r="273">
@@ -2778,7 +2687,7 @@
         <v>272.0</v>
       </c>
       <c r="B273" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="274">
@@ -2786,7 +2695,7 @@
         <v>273.0</v>
       </c>
       <c r="B274" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.28E7</v>
       </c>
     </row>
     <row r="275">
@@ -2794,7 +2703,7 @@
         <v>274.0</v>
       </c>
       <c r="B275" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.28E7</v>
       </c>
     </row>
     <row r="276">
@@ -2802,7 +2711,7 @@
         <v>275.0</v>
       </c>
       <c r="B276" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="277">
@@ -2810,7 +2719,7 @@
         <v>276.0</v>
       </c>
       <c r="B277" t="n" s="0">
-        <v>2.42E7</v>
+        <v>5.05E7</v>
       </c>
     </row>
     <row r="278">
@@ -2818,7 +2727,7 @@
         <v>277.0</v>
       </c>
       <c r="B278" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.285E7</v>
       </c>
     </row>
     <row r="279">
@@ -2826,7 +2735,7 @@
         <v>278.0</v>
       </c>
       <c r="B279" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="280">
@@ -2834,7 +2743,7 @@
         <v>279.0</v>
       </c>
       <c r="B280" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.19E7</v>
       </c>
     </row>
     <row r="281">
@@ -2842,7 +2751,7 @@
         <v>280.0</v>
       </c>
       <c r="B281" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.33E7</v>
       </c>
     </row>
     <row r="282">
@@ -2850,7 +2759,7 @@
         <v>281.0</v>
       </c>
       <c r="B282" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.28E7</v>
       </c>
     </row>
     <row r="283">
@@ -2858,7 +2767,7 @@
         <v>282.0</v>
       </c>
       <c r="B283" t="n" s="0">
-        <v>2.42E7</v>
+        <v>6.77E7</v>
       </c>
     </row>
     <row r="284">
@@ -2866,7 +2775,7 @@
         <v>283.0</v>
       </c>
       <c r="B284" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.28E7</v>
       </c>
     </row>
     <row r="285">
@@ -2874,7 +2783,7 @@
         <v>284.0</v>
       </c>
       <c r="B285" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.28E7</v>
       </c>
     </row>
     <row r="286">
@@ -2882,7 +2791,7 @@
         <v>285.0</v>
       </c>
       <c r="B286" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.375E7</v>
       </c>
     </row>
     <row r="287">
@@ -2890,7 +2799,7 @@
         <v>286.0</v>
       </c>
       <c r="B287" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.375E7</v>
       </c>
     </row>
     <row r="288">
@@ -2898,7 +2807,7 @@
         <v>287.0</v>
       </c>
       <c r="B288" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.375E7</v>
       </c>
     </row>
     <row r="289">
@@ -2906,7 +2815,7 @@
         <v>288.0</v>
       </c>
       <c r="B289" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.375E7</v>
       </c>
     </row>
     <row r="290">
@@ -2914,7 +2823,7 @@
         <v>289.0</v>
       </c>
       <c r="B290" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.375E7</v>
       </c>
     </row>
     <row r="291">
@@ -2922,7 +2831,7 @@
         <v>290.0</v>
       </c>
       <c r="B291" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.375E7</v>
       </c>
     </row>
     <row r="292">
@@ -2930,7 +2839,7 @@
         <v>291.0</v>
       </c>
       <c r="B292" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.375E7</v>
       </c>
     </row>
     <row r="293">
@@ -2938,7 +2847,7 @@
         <v>292.0</v>
       </c>
       <c r="B293" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.375E7</v>
       </c>
     </row>
     <row r="294">
@@ -2946,7 +2855,7 @@
         <v>293.0</v>
       </c>
       <c r="B294" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.375E7</v>
       </c>
     </row>
     <row r="295">
@@ -2954,7 +2863,7 @@
         <v>294.0</v>
       </c>
       <c r="B295" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.28E7</v>
       </c>
     </row>
     <row r="296">
@@ -2962,7 +2871,7 @@
         <v>295.0</v>
       </c>
       <c r="B296" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.28E7</v>
       </c>
     </row>
     <row r="297">
@@ -2970,7 +2879,7 @@
         <v>296.0</v>
       </c>
       <c r="B297" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.33E7</v>
       </c>
     </row>
     <row r="298">
@@ -2978,7 +2887,7 @@
         <v>297.0</v>
       </c>
       <c r="B298" t="n" s="0">
-        <v>2.42E7</v>
+        <v>3.375E7</v>
       </c>
     </row>
     <row r="299">
@@ -2986,7 +2895,7 @@
         <v>298.0</v>
       </c>
       <c r="B299" t="n" s="0">
-        <v>2.42E7</v>
+        <v>4.14E7</v>
       </c>
     </row>
     <row r="300">
@@ -2994,7 +2903,7 @@
         <v>299.0</v>
       </c>
       <c r="B300" t="n" s="0">
-        <v>2.42E7</v>
+        <v>6.77E7</v>
       </c>
     </row>
     <row r="301">
@@ -3002,7 +2911,7 @@
         <v>300.0</v>
       </c>
       <c r="B301" t="n" s="0">
-        <v>2.42E7</v>
+        <v>6.77E7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>